<commit_message>
Updated POL_grids_kan model - 2025-12-05 16:32
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{541415CF-D844-4E04-8F57-532D08AFEAF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F0F35DF8-A1E1-4025-98E4-28DD9A77E3AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29302,7 +29302,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00AB7EAD-C8F7-482F-84AD-305F1EB21891}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C59A7B34-A1A5-48BC-B858-34CB8AF7D426}">
   <dimension ref="B9:H285"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -34462,7 +34462,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E334DCD6-890D-4CC5-B8BA-5B4D94C3984E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08F9D403-063A-4EF5-B6C0-2805D8D291F3}">
   <dimension ref="B9:L285"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_kan model - 2026-06-05 17:25
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{731C1EA2-0D44-4FF1-B39F-9004F18ACD0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{63E7D933-CAED-4B86-9A6F-70FB68D1AAF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4450,7 +4450,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{548BE81A-C8E8-4305-A6A6-32F44D5567B3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F60670B4-7FE5-4533-89B2-57A418C7F62C}">
   <dimension ref="B9:H285"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -30132,7 +30132,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3F94D5A-203B-4EA9-AAE6-66EC47BDEABE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B28B4809-9393-4FF0-8E58-70B539E7ED30}">
   <dimension ref="B9:L285"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_kan model - 2026-06-08 18:02
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{63E7D933-CAED-4B86-9A6F-70FB68D1AAF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FC23EA4F-124A-43AE-A2A9-BF9FF53CBF2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4450,7 +4450,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F60670B4-7FE5-4533-89B2-57A418C7F62C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EB1077C-72D2-4EB4-A404-4AA342C153CF}">
   <dimension ref="B9:H285"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -30132,7 +30132,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B28B4809-9393-4FF0-8E58-70B539E7ED30}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE9D65A2-3E8B-424C-AFEE-412FA0D02070}">
   <dimension ref="B9:L285"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_kan model - 2026-06-08 18:31
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FC23EA4F-124A-43AE-A2A9-BF9FF53CBF2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F21FE918-2525-4071-BE11-2C13FB8D17A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4450,7 +4450,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EB1077C-72D2-4EB4-A404-4AA342C153CF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91A5045C-A983-4FBB-9647-D50504DB73E3}">
   <dimension ref="B9:H285"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -30132,7 +30132,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE9D65A2-3E8B-424C-AFEE-412FA0D02070}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E03CF7CB-0BB1-4B05-880B-F898A2AA9566}">
   <dimension ref="B9:L285"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_kan model - 2026-06-09 15:52
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{78637BD8-38F9-4E4B-B041-B339CF03966D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0CE24622-84B5-4A49-886F-9D83C2AA6400}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4280,7 +4280,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CDD08C4A-A30B-7B00-9FF5-BA7CFDC924F4}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9F216277-49B3-8AEA-14B7-5D8F1548DA26}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4335,7 +4335,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8230E076-48C2-A365-6B1A-B51BAA96A7EA}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{104F1A72-28A0-C0AF-7F47-D7C0D4BCE6FC}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4656,7 +4656,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E559C0D1-F238-42C7-86A5-88780DF9C738}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F06CDC2-7CE3-44BA-8DEC-8A8539B5D01D}">
   <dimension ref="A1:H285"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -30411,7 +30411,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D5B52BB-E6D2-4774-8007-AD27380B46B6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{158A455D-3200-4B64-A4D3-217EAEB13E53}">
   <dimension ref="A1:L285"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>

</xml_diff>

<commit_message>
Updated POL_grids_kan model - 2026-06-12 13:27
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{05ED7120-721C-4715-AA25-DB6C7C0B0E14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A5308D7-9C5C-4300-8F3E-23781F42301C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4450,7 +4450,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F831FFB-1B86-4C1B-91E8-135B4FC8C4C3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36EB9973-006D-4C3B-B246-F624C02A7585}">
   <dimension ref="B9:H285"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -30132,7 +30132,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52762E74-B7FF-49AE-B6E5-3C17A29B241F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFB64FFD-757B-4676-BE19-55E649E6BC80}">
   <dimension ref="B9:L285"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_kan model - 2026-06-12 14:16
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A5308D7-9C5C-4300-8F3E-23781F42301C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{93001361-F289-43B2-A5C5-597204E1FE02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4450,7 +4450,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36EB9973-006D-4C3B-B246-F624C02A7585}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B2F026D-B2FE-4B7A-A654-EB510175C638}">
   <dimension ref="B9:H285"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -30132,7 +30132,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFB64FFD-757B-4676-BE19-55E649E6BC80}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{807198DE-301E-42F8-812C-4C7217351240}">
   <dimension ref="B9:L285"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_kan model - 2026-06-12 14:51
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{93001361-F289-43B2-A5C5-597204E1FE02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EC3FBF61-EC17-4FD7-A297-1A877E9239C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4450,7 +4450,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B2F026D-B2FE-4B7A-A654-EB510175C638}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED425EC8-34E4-40A7-8E63-5FA7B79DCF0B}">
   <dimension ref="B9:H285"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -30132,7 +30132,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{807198DE-301E-42F8-812C-4C7217351240}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CB3EFE0-322A-4977-9796-DFCF4BB22297}">
   <dimension ref="B9:L285"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>